<commit_message>
audit: correct CI/CD dashboard metrics, update findings spreadsheet status to Resolved, and separate security test cases from scan rules
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/findings.xlsx
+++ b/Vulnerability Test Results/findings.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>

</xml_diff>